<commit_message>
Enable downloading Master format with live data for editing and re-uploading
</commit_message>
<xml_diff>
--- a/static/Employee_Master_Import_Template.xlsx
+++ b/static/Employee_Master_Import_Template.xlsx
@@ -26,17 +26,17 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Segoe UI"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -45,14 +45,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00800000"/>
-        <bgColor rgb="00800000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
+        <fgColor rgb="001E3A8A"/>
+        <bgColor rgb="001E3A8A"/>
       </patternFill>
     </fill>
   </fills>
@@ -66,16 +60,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="00D1D5DB"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="00D1D5DB"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="00D1D5DB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="00D1D5DB"/>
       </bottom>
     </border>
   </borders>
@@ -84,16 +78,16 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -461,39 +455,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA4"/>
+  <dimension ref="A1:AB2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="15" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="26" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="24" customWidth="1" min="20" max="20"/>
-    <col width="21" customWidth="1" min="21" max="21"/>
-    <col width="19" customWidth="1" min="22" max="22"/>
-    <col width="16" customWidth="1" min="23" max="23"/>
-    <col width="14" customWidth="1" min="24" max="24"/>
-    <col width="15" customWidth="1" min="25" max="25"/>
-    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="15" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
     <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Emp_No</t>
@@ -504,139 +499,144 @@
           <t>Employee_Name</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Employee_Type</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Payroll_Category</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Designation</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Grade</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>DOJ</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>DOB</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Father_Name</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Bank_Acc_No</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Bank_IFSC</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>UAN_No</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ESI_No</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Phone_Number</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Email_ID</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Fixed_Gross</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Basic_DA</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>HRA</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Conveyance_Allowance</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Washing_Allowance</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Other_Allowance</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Per_Day_Wage</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>OT_Rate</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>PF_Eligible</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>ESI_Eligible</t>
         </is>
       </c>
-      <c r="AA1" s="2" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>LIC</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+    <row r="2" ht="21" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>1001</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Rajesh Kumar</t>
         </is>
@@ -651,12 +651,12 @@
           <t>PF_ESI</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>CNC Operator</t>
         </is>
@@ -668,60 +668,62 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
           <t>2024-01-15</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>1995-08-20</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Ramesh Kumar</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>918273645012</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>SBIN0001234</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>100918273645</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>3109182736</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
-        <is>
-          <t>9876543210</t>
-        </is>
-      </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>+919876543210</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>rajesh@example.com</t>
         </is>
       </c>
-      <c r="Q2" s="4" t="n">
+      <c r="R2" s="4" t="n">
         <v>25000</v>
       </c>
-      <c r="R2" s="4" t="n">
+      <c r="S2" s="4" t="n">
         <v>12500</v>
       </c>
-      <c r="S2" s="4" t="n">
+      <c r="T2" s="4" t="n">
         <v>5000</v>
-      </c>
-      <c r="T2" s="4" t="n">
-        <v>2500</v>
       </c>
       <c r="U2" s="4" t="n">
         <v>2500</v>
@@ -730,253 +732,26 @@
         <v>2500</v>
       </c>
       <c r="W2" s="4" t="n">
+        <v>2500</v>
+      </c>
+      <c r="X2" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="X2" s="4" t="n">
+      <c r="Y2" s="4" t="n">
         <v>81.25</v>
       </c>
-      <c r="Y2" s="3" t="inlineStr">
+      <c r="Z2" s="3" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="Z2" s="3" t="inlineStr">
+      <c r="AA2" s="3" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="AA2" s="4" t="n">
+      <c r="AB2" s="4" t="n">
         <v>500</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>1002</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Suresh M</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>WORKER</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>PF_ESI</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Assembly</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Fitter</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Grade B</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>2024-02-01</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>1998-11-10</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Murugan</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>918273645013</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>IOBA0001234</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>100918273646</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>3109182737</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="inlineStr">
-        <is>
-          <t>9876543211</t>
-        </is>
-      </c>
-      <c r="P3" s="3" t="inlineStr">
-        <is>
-          <t>suresh@example.com</t>
-        </is>
-      </c>
-      <c r="Q3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W3" s="4" t="n">
-        <v>650</v>
-      </c>
-      <c r="X3" s="4" t="n">
-        <v>56.25</v>
-      </c>
-      <c r="Y3" s="3" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="Z3" s="3" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="AA3" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>1003</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Anitha R</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>STAFF</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>NAPS</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Quality</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Inspector</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Apprentice</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>2024-03-10</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>2001-04-05</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>Ramasamy</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>918273645014</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>HDFC0001234</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr"/>
-      <c r="N4" s="3" t="inlineStr"/>
-      <c r="O4" s="3" t="inlineStr">
-        <is>
-          <t>9876543212</t>
-        </is>
-      </c>
-      <c r="P4" s="3" t="inlineStr">
-        <is>
-          <t>anitha@example.com</t>
-        </is>
-      </c>
-      <c r="Q4" s="4" t="n">
-        <v>15000</v>
-      </c>
-      <c r="R4" s="4" t="n">
-        <v>7500</v>
-      </c>
-      <c r="S4" s="4" t="n">
-        <v>3000</v>
-      </c>
-      <c r="T4" s="4" t="n">
-        <v>1500</v>
-      </c>
-      <c r="U4" s="4" t="n">
-        <v>1500</v>
-      </c>
-      <c r="V4" s="4" t="n">
-        <v>1500</v>
-      </c>
-      <c r="W4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X4" s="4" t="n">
-        <v>56.25</v>
-      </c>
-      <c r="Y4" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="Z4" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="AA4" s="4" t="n">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>